<commit_message>
Regenerar comparativa superficie adicional con reparto real por titular
comparativa_300_vs_300_superficie_adicional.xlsx (sobrescrito) y su script:
la superficie externa (vinedo, frutales, horticolas) se reparte por
territorio segun el dato REAL por titular (superficie de cultivo
declarada en cada TH), no por proporcion SIGPAC, que sobrecargaba Araba.
Total externas por categoria y Euskadi sin cambios; solo cambia el
reparto entre territorios (Cuadro 2). Validado contra A y B.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparativa_300_vs_300_superficie_adicional.xlsx
+++ b/comparativa_300_vs_300_superficie_adicional.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>CUADRO 1 — Nº de beneficiarios (solo beneficiarios existentes)</t>
+          <t>CUADRO 1 — Nº de beneficiarios (existentes)</t>
         </is>
       </c>
     </row>
@@ -548,10 +548,10 @@
         <v>94487.59</v>
       </c>
       <c r="C10" t="n">
-        <v>97606.64999999999</v>
+        <v>97141.5</v>
       </c>
       <c r="D10" t="n">
-        <v>-3119.06</v>
+        <v>-2653.91</v>
       </c>
     </row>
     <row r="11">
@@ -564,10 +564,10 @@
         <v>30734.97</v>
       </c>
       <c r="C11" t="n">
-        <v>32647.32</v>
+        <v>33399.2</v>
       </c>
       <c r="D11" t="n">
-        <v>-1912.35</v>
+        <v>-2664.23</v>
       </c>
     </row>
     <row r="12">
@@ -580,10 +580,10 @@
         <v>27781.65</v>
       </c>
       <c r="C12" t="n">
-        <v>29048.96</v>
+        <v>28762.22</v>
       </c>
       <c r="D12" t="n">
-        <v>-1267.31</v>
+        <v>-980.5700000000001</v>
       </c>
     </row>
     <row r="13">
@@ -698,7 +698,149 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NOTA: Este escenario refleja SOLO el efecto sobre las explotaciones existentes (no se añaden nuevas). La superficie adicional incorporada (viñedo, frutales, hortícolas) reduce ligeramente el importe medio del existente al ampliar el denominador. ADVERTENCIA: si se incorporaran las nuevas explotaciones que generaría esa superficie (~6.124 estimadas, sobre todo frutales y hortícolas de tamaño muy pequeño), el importe medio por explotación caería con fuerza (en Euskadi, de ~6.423 € a ~3.400 €), NO por reducción del presupuesto (constante: 42.353.115,52 €) sino por repartirse entre muchas más explotaciones pequeñas.</t>
+          <t>REPARTO de la superficie incorporada por categoría y territorio (dato real por titular)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Método</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Araba</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Gipuzkoa</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Bizkaia</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Viñedo y Txakoli</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Dato real por titular</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2448.38</v>
+      </c>
+      <c r="D24" t="n">
+        <v>121.28</v>
+      </c>
+      <c r="E24" t="n">
+        <v>109.68</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2679.34</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Frutales y frutos secos</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Dato real por titular</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>190.58</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2428.66</v>
+      </c>
+      <c r="E25" t="n">
+        <v>732.65</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3351.89</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hortícolas</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Dato real por titular</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>14.95</v>
+      </c>
+      <c r="D26" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="E26" t="n">
+        <v>138.24</v>
+      </c>
+      <c r="F26" t="n">
+        <v>267.49</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TOTAL externas</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2653.91</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2664.23</v>
+      </c>
+      <c r="E27" t="n">
+        <v>980.5700000000001</v>
+      </c>
+      <c r="F27" t="n">
+        <v>6298.72</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>NOTA:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>NOTA 1 — La superficie ABRS sin derecho NO se suma en B: ya está incluida en la superficie activada del Escenario A (153.004,21 ha). En la base &gt;300 asciende a 13.936,08 ha. En B solo se incorporan los cultivos externos (6.298,72 ha).  NOTA 2 — Las externas se reparten por territorio según el DATO REAL POR TITULAR (superficie de cultivo declarada en cada TH), no por proporción SIGPAC.  NOTA 3 — Los cuadros mantienen las explotaciones EXISTENTES. Esa superficie generaría ~6.124 explotaciones teóricas nuevas (sobre todo frutales y hortícolas de tamaño muy pequeño); si se contaran, el importe medio en Euskadi caería de ~6.423,26 € a ~3.399,95 €, por repartir el mismo presupuesto (42.353.115,52 €) entre muchas más explotaciones.</t>
         </is>
       </c>
     </row>

</xml_diff>